<commit_message>
Update factory layout Excel template
</commit_message>
<xml_diff>
--- a/backend/app/templates/factory_layout_template.xlsx
+++ b/backend/app/templates/factory_layout_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16b59dc5d76a24f7/Desktop/회사 문서/연구소/공장 배치/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="451" documentId="11_0EEEB546568656891A6EEC37D73FD0AA7EDE8998" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0AF5DCA-CE1D-4965-9F7A-A29D0C7960BD}"/>
+  <xr:revisionPtr revIDLastSave="499" documentId="11_0EEEB546568656891A6EEC37D73FD0AA7EDE8998" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C0324F0-60A2-434B-A715-5E739A3304E1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,143 +89,139 @@
   </si>
   <si>
     <t>조립동</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>제관동</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>가공동</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>기계</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-12</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-11</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-10</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>기둥</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-21</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-17</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-16</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-15</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-01</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-02</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-03</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-04</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-05</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-06</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-07</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-08</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-09</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-10</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-11</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-12</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-13</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-14</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B-15</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>B구역</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A구역</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>C구역</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>C-06</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>C-07</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>사무동</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>공장 배치도</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-01</t>
-    <phoneticPr fontId="10" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>A-02</t>
@@ -250,13 +246,17 @@
   </si>
   <si>
     <t>A-09</t>
+  </si>
+  <si>
+    <t>공장 배치도 (Lay Out)</t>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -295,14 +295,6 @@
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Malgun Gothic"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF006B23"/>
       <name val="Malgun Gothic"/>
       <family val="3"/>
       <charset val="129"/>
@@ -394,6 +386,38 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <b/>
+      <sz val="17"/>
+      <color rgb="FF123047"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="17"/>
+      <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="30"/>
+      <color rgb="FF123047"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -904,15 +928,15 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -941,30 +965,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -977,157 +980,127 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="23" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="23" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="25" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="25" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="22" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="24" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="27" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="21" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="22" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="22" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="23" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="27" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1136,77 +1109,140 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="21" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="22" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="24" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="27" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="39" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="40" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="38" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1394,18 +1430,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:26" ht="24" customHeight="1">
-      <c r="A2" s="29"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -1422,20 +1458,20 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="24" customHeight="1">
-      <c r="A3" s="29"/>
-      <c r="B3" s="98" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="102" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -1452,18 +1488,18 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="24" customHeight="1">
-      <c r="A4" s="29"/>
-      <c r="B4" s="98"/>
-      <c r="C4" s="98"/>
-      <c r="D4" s="98"/>
-      <c r="E4" s="98"/>
-      <c r="F4" s="98"/>
-      <c r="G4" s="98"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -1481,17 +1517,17 @@
     </row>
     <row r="5" spans="1:26" ht="24" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="98"/>
-      <c r="C5" s="98"/>
-      <c r="D5" s="98"/>
-      <c r="E5" s="98"/>
-      <c r="F5" s="98"/>
-      <c r="G5" s="98"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -1541,7 +1577,7 @@
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="26"/>
+      <c r="F7" s="19"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1569,86 +1605,86 @@
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="35" t="s">
+      <c r="F8" s="23"/>
+      <c r="G8" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="H8" s="35"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
-      <c r="S8" s="30"/>
-      <c r="T8" s="30"/>
-      <c r="U8" s="30"/>
-      <c r="V8" s="30"/>
-      <c r="W8" s="30"/>
-      <c r="X8" s="30"/>
-      <c r="Y8" s="67"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="23"/>
+      <c r="R8" s="23"/>
+      <c r="S8" s="23"/>
+      <c r="T8" s="23"/>
+      <c r="U8" s="23"/>
+      <c r="V8" s="23"/>
+      <c r="W8" s="23"/>
+      <c r="X8" s="23"/>
+      <c r="Y8" s="52"/>
       <c r="Z8" s="6"/>
     </row>
     <row r="9" spans="1:26" ht="24" customHeight="1" thickBot="1">
       <c r="A9" s="5"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="73" t="s">
+      <c r="B9" s="65"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="68" t="s">
+      <c r="G9" s="13"/>
+      <c r="H9" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="69"/>
-      <c r="J9" s="69"/>
-      <c r="K9" s="70"/>
-      <c r="L9" s="11" t="s">
+      <c r="I9" s="54"/>
+      <c r="J9" s="54"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="83" t="s">
         <v>56</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="N9" s="83" t="s">
         <v>57</v>
       </c>
-      <c r="N9" s="11" t="s">
+      <c r="O9" s="83" t="s">
         <v>58</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="P9" s="83" t="s">
         <v>59</v>
       </c>
-      <c r="P9" s="11" t="s">
+      <c r="Q9" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="R9" s="83" t="s">
         <v>61</v>
       </c>
-      <c r="R9" s="11" t="s">
+      <c r="S9" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="S9" s="11" t="s">
+      <c r="T9" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="T9" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="U9" s="11" t="s">
+      <c r="U9" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="11" t="s">
+      <c r="V9" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="W9" s="11" t="s">
+      <c r="W9" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="X9" s="11" t="s">
+      <c r="X9" s="83" t="s">
         <v>29</v>
       </c>
-      <c r="Y9" s="67"/>
+      <c r="Y9" s="52"/>
       <c r="Z9" s="6"/>
     </row>
     <row r="10" spans="1:26" ht="24" customHeight="1" thickBot="1">
@@ -1657,7 +1693,7 @@
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="74"/>
+      <c r="F10" s="57"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
@@ -1675,10 +1711,10 @@
       <c r="U10" s="9"/>
       <c r="V10" s="9"/>
       <c r="W10" s="9"/>
-      <c r="X10" s="11" t="s">
+      <c r="X10" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="Y10" s="67"/>
+      <c r="Y10" s="52"/>
       <c r="Z10" s="6"/>
     </row>
     <row r="11" spans="1:26" ht="24" customHeight="1" thickBot="1">
@@ -1687,7 +1723,7 @@
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
-      <c r="F11" s="21"/>
+      <c r="F11" s="14"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
@@ -1705,10 +1741,10 @@
       <c r="U11" s="9"/>
       <c r="V11" s="9"/>
       <c r="W11" s="9"/>
-      <c r="X11" s="11" t="s">
+      <c r="X11" s="83" t="s">
         <v>4</v>
       </c>
-      <c r="Y11" s="67"/>
+      <c r="Y11" s="52"/>
       <c r="Z11" s="6"/>
     </row>
     <row r="12" spans="1:26" ht="24" customHeight="1" thickBot="1">
@@ -1717,7 +1753,7 @@
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="83" t="s">
         <v>1</v>
       </c>
       <c r="G12" s="9"/>
@@ -1737,21 +1773,21 @@
       <c r="U12" s="9"/>
       <c r="V12" s="9"/>
       <c r="W12" s="9"/>
-      <c r="X12" s="71" t="s">
+      <c r="X12" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="Y12" s="67"/>
+      <c r="Y12" s="52"/>
       <c r="Z12" s="6"/>
     </row>
     <row r="13" spans="1:26" ht="24" customHeight="1" thickBot="1">
       <c r="A13" s="5"/>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="36"/>
+      <c r="C13" s="70"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="83" t="s">
         <v>3</v>
       </c>
       <c r="G13" s="9"/>
@@ -1771,8 +1807,8 @@
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
       <c r="W13" s="9"/>
-      <c r="X13" s="72"/>
-      <c r="Y13" s="67"/>
+      <c r="X13" s="85"/>
+      <c r="Y13" s="52"/>
       <c r="Z13" s="6"/>
     </row>
     <row r="14" spans="1:26" ht="24" customHeight="1" thickBot="1">
@@ -1781,394 +1817,394 @@
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="83" t="s">
         <v>29</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="83" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="75" t="s">
+      <c r="I14" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="J14" s="76"/>
-      <c r="K14" s="11" t="s">
+      <c r="J14" s="90"/>
+      <c r="K14" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="L14" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="M14" s="11" t="s">
+      <c r="M14" s="83" t="s">
         <v>9</v>
       </c>
-      <c r="N14" s="16" t="s">
+      <c r="N14" s="88" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="77" t="s">
+      <c r="O14" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="P14" s="78"/>
-      <c r="Q14" s="11" t="s">
+      <c r="P14" s="87"/>
+      <c r="Q14" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="R14" s="11" t="s">
+      <c r="R14" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="S14" s="11" t="s">
+      <c r="S14" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="T14" s="11" t="s">
+      <c r="T14" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="U14" s="77" t="s">
+      <c r="U14" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="V14" s="78"/>
-      <c r="W14" s="11" t="s">
+      <c r="V14" s="87"/>
+      <c r="W14" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="X14" s="11" t="s">
+      <c r="X14" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="Y14" s="67"/>
+      <c r="Y14" s="52"/>
       <c r="Z14" s="6"/>
     </row>
     <row r="15" spans="1:26" ht="24" customHeight="1">
       <c r="A15" s="5"/>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="91" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="40" t="s">
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="58" t="s">
+      <c r="F15" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="G15" s="59"/>
-      <c r="H15" s="59"/>
-      <c r="I15" s="59"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="89" t="s">
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="N15" s="90"/>
-      <c r="O15" s="90"/>
-      <c r="P15" s="90"/>
-      <c r="Q15" s="90"/>
-      <c r="R15" s="91"/>
-      <c r="S15" s="45" t="s">
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="35"/>
+      <c r="R15" s="36"/>
+      <c r="S15" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="T15" s="46"/>
-      <c r="U15" s="46"/>
-      <c r="V15" s="46"/>
-      <c r="W15" s="46"/>
-      <c r="X15" s="46"/>
-      <c r="Y15" s="67"/>
+      <c r="T15" s="78"/>
+      <c r="U15" s="78"/>
+      <c r="V15" s="78"/>
+      <c r="W15" s="78"/>
+      <c r="X15" s="78"/>
+      <c r="Y15" s="52"/>
       <c r="Z15" s="6"/>
     </row>
     <row r="16" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A16" s="5"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="62"/>
-      <c r="H16" s="62"/>
-      <c r="I16" s="62"/>
-      <c r="J16" s="62"/>
-      <c r="K16" s="62"/>
-      <c r="L16" s="63"/>
-      <c r="M16" s="92"/>
-      <c r="N16" s="93"/>
-      <c r="O16" s="93"/>
-      <c r="P16" s="93"/>
-      <c r="Q16" s="93"/>
-      <c r="R16" s="94"/>
-      <c r="S16" s="47"/>
-      <c r="T16" s="48"/>
-      <c r="U16" s="48"/>
-      <c r="V16" s="48"/>
-      <c r="W16" s="48"/>
-      <c r="X16" s="48"/>
-      <c r="Y16" s="67"/>
+      <c r="B16" s="92"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="92"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="47"/>
+      <c r="K16" s="47"/>
+      <c r="L16" s="48"/>
+      <c r="M16" s="37"/>
+      <c r="N16" s="38"/>
+      <c r="O16" s="38"/>
+      <c r="P16" s="38"/>
+      <c r="Q16" s="38"/>
+      <c r="R16" s="39"/>
+      <c r="S16" s="79"/>
+      <c r="T16" s="80"/>
+      <c r="U16" s="80"/>
+      <c r="V16" s="80"/>
+      <c r="W16" s="80"/>
+      <c r="X16" s="80"/>
+      <c r="Y16" s="52"/>
       <c r="Z16" s="6"/>
     </row>
     <row r="17" spans="1:26" ht="26" customHeight="1">
       <c r="A17" s="5"/>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="91" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="40" t="s">
+      <c r="C17" s="75"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="61"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="62"/>
-      <c r="K17" s="62"/>
-      <c r="L17" s="63"/>
-      <c r="M17" s="92"/>
-      <c r="N17" s="93"/>
-      <c r="O17" s="93"/>
-      <c r="P17" s="93"/>
-      <c r="Q17" s="93"/>
-      <c r="R17" s="94"/>
-      <c r="S17" s="47"/>
-      <c r="T17" s="48"/>
-      <c r="U17" s="48"/>
-      <c r="V17" s="48"/>
-      <c r="W17" s="48"/>
-      <c r="X17" s="48"/>
-      <c r="Y17" s="67"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="47"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="47"/>
+      <c r="L17" s="48"/>
+      <c r="M17" s="37"/>
+      <c r="N17" s="38"/>
+      <c r="O17" s="38"/>
+      <c r="P17" s="38"/>
+      <c r="Q17" s="38"/>
+      <c r="R17" s="39"/>
+      <c r="S17" s="79"/>
+      <c r="T17" s="80"/>
+      <c r="U17" s="80"/>
+      <c r="V17" s="80"/>
+      <c r="W17" s="80"/>
+      <c r="X17" s="80"/>
+      <c r="Y17" s="52"/>
       <c r="Z17" s="6"/>
     </row>
     <row r="18" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A18" s="5"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="62"/>
-      <c r="H18" s="62"/>
-      <c r="I18" s="62"/>
-      <c r="J18" s="62"/>
-      <c r="K18" s="62"/>
-      <c r="L18" s="63"/>
-      <c r="M18" s="92"/>
-      <c r="N18" s="93"/>
-      <c r="O18" s="93"/>
-      <c r="P18" s="93"/>
-      <c r="Q18" s="93"/>
-      <c r="R18" s="94"/>
-      <c r="S18" s="47"/>
-      <c r="T18" s="48"/>
-      <c r="U18" s="48"/>
-      <c r="V18" s="48"/>
-      <c r="W18" s="48"/>
-      <c r="X18" s="48"/>
-      <c r="Y18" s="67"/>
+      <c r="B18" s="92"/>
+      <c r="C18" s="75"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="92"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="47"/>
+      <c r="H18" s="47"/>
+      <c r="I18" s="47"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="47"/>
+      <c r="L18" s="48"/>
+      <c r="M18" s="37"/>
+      <c r="N18" s="38"/>
+      <c r="O18" s="38"/>
+      <c r="P18" s="38"/>
+      <c r="Q18" s="38"/>
+      <c r="R18" s="39"/>
+      <c r="S18" s="79"/>
+      <c r="T18" s="80"/>
+      <c r="U18" s="80"/>
+      <c r="V18" s="80"/>
+      <c r="W18" s="80"/>
+      <c r="X18" s="80"/>
+      <c r="Y18" s="52"/>
       <c r="Z18" s="6"/>
     </row>
     <row r="19" spans="1:26" ht="26" customHeight="1">
       <c r="A19" s="5"/>
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="40" t="s">
+      <c r="C19" s="75"/>
+      <c r="D19" s="75"/>
+      <c r="E19" s="91" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="61"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="62"/>
-      <c r="K19" s="62"/>
-      <c r="L19" s="63"/>
-      <c r="M19" s="92"/>
-      <c r="N19" s="93"/>
-      <c r="O19" s="93"/>
-      <c r="P19" s="93"/>
-      <c r="Q19" s="93"/>
-      <c r="R19" s="94"/>
-      <c r="S19" s="47"/>
-      <c r="T19" s="48"/>
-      <c r="U19" s="48"/>
-      <c r="V19" s="48"/>
-      <c r="W19" s="48"/>
-      <c r="X19" s="48"/>
-      <c r="Y19" s="67"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="48"/>
+      <c r="M19" s="37"/>
+      <c r="N19" s="38"/>
+      <c r="O19" s="38"/>
+      <c r="P19" s="38"/>
+      <c r="Q19" s="38"/>
+      <c r="R19" s="39"/>
+      <c r="S19" s="79"/>
+      <c r="T19" s="80"/>
+      <c r="U19" s="80"/>
+      <c r="V19" s="80"/>
+      <c r="W19" s="80"/>
+      <c r="X19" s="80"/>
+      <c r="Y19" s="52"/>
       <c r="Z19" s="6"/>
     </row>
     <row r="20" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A20" s="5"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="62"/>
-      <c r="H20" s="62"/>
-      <c r="I20" s="62"/>
-      <c r="J20" s="62"/>
-      <c r="K20" s="62"/>
-      <c r="L20" s="63"/>
-      <c r="M20" s="92"/>
-      <c r="N20" s="93"/>
-      <c r="O20" s="93"/>
-      <c r="P20" s="93"/>
-      <c r="Q20" s="93"/>
-      <c r="R20" s="94"/>
-      <c r="S20" s="47"/>
-      <c r="T20" s="48"/>
-      <c r="U20" s="48"/>
-      <c r="V20" s="48"/>
-      <c r="W20" s="48"/>
-      <c r="X20" s="48"/>
-      <c r="Y20" s="67"/>
+      <c r="B20" s="92"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="75"/>
+      <c r="E20" s="92"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="47"/>
+      <c r="K20" s="47"/>
+      <c r="L20" s="48"/>
+      <c r="M20" s="37"/>
+      <c r="N20" s="38"/>
+      <c r="O20" s="38"/>
+      <c r="P20" s="38"/>
+      <c r="Q20" s="38"/>
+      <c r="R20" s="39"/>
+      <c r="S20" s="79"/>
+      <c r="T20" s="80"/>
+      <c r="U20" s="80"/>
+      <c r="V20" s="80"/>
+      <c r="W20" s="80"/>
+      <c r="X20" s="80"/>
+      <c r="Y20" s="52"/>
       <c r="Z20" s="6"/>
     </row>
     <row r="21" spans="1:26" ht="26" customHeight="1">
       <c r="A21" s="5"/>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="91" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="40" t="s">
+      <c r="C21" s="75"/>
+      <c r="D21" s="75"/>
+      <c r="E21" s="91" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="61"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="62"/>
-      <c r="J21" s="62"/>
-      <c r="K21" s="62"/>
-      <c r="L21" s="63"/>
-      <c r="M21" s="92"/>
-      <c r="N21" s="93"/>
-      <c r="O21" s="93"/>
-      <c r="P21" s="93"/>
-      <c r="Q21" s="93"/>
-      <c r="R21" s="94"/>
-      <c r="S21" s="47"/>
-      <c r="T21" s="48"/>
-      <c r="U21" s="48"/>
-      <c r="V21" s="48"/>
-      <c r="W21" s="48"/>
-      <c r="X21" s="48"/>
-      <c r="Y21" s="67"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="47"/>
+      <c r="J21" s="47"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="48"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="38"/>
+      <c r="O21" s="38"/>
+      <c r="P21" s="38"/>
+      <c r="Q21" s="38"/>
+      <c r="R21" s="39"/>
+      <c r="S21" s="79"/>
+      <c r="T21" s="80"/>
+      <c r="U21" s="80"/>
+      <c r="V21" s="80"/>
+      <c r="W21" s="80"/>
+      <c r="X21" s="80"/>
+      <c r="Y21" s="52"/>
       <c r="Z21" s="6"/>
     </row>
     <row r="22" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A22" s="5"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="62"/>
-      <c r="H22" s="62"/>
-      <c r="I22" s="62"/>
-      <c r="J22" s="62"/>
-      <c r="K22" s="62"/>
-      <c r="L22" s="63"/>
-      <c r="M22" s="92"/>
-      <c r="N22" s="93"/>
-      <c r="O22" s="93"/>
-      <c r="P22" s="93"/>
-      <c r="Q22" s="93"/>
-      <c r="R22" s="94"/>
-      <c r="S22" s="47"/>
-      <c r="T22" s="48"/>
-      <c r="U22" s="48"/>
-      <c r="V22" s="48"/>
-      <c r="W22" s="48"/>
-      <c r="X22" s="48"/>
-      <c r="Y22" s="67"/>
+      <c r="B22" s="92"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="92"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="48"/>
+      <c r="M22" s="37"/>
+      <c r="N22" s="38"/>
+      <c r="O22" s="38"/>
+      <c r="P22" s="38"/>
+      <c r="Q22" s="38"/>
+      <c r="R22" s="39"/>
+      <c r="S22" s="79"/>
+      <c r="T22" s="80"/>
+      <c r="U22" s="80"/>
+      <c r="V22" s="80"/>
+      <c r="W22" s="80"/>
+      <c r="X22" s="80"/>
+      <c r="Y22" s="52"/>
       <c r="Z22" s="6"/>
     </row>
     <row r="23" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A23" s="5"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="40" t="s">
+      <c r="B23" s="11"/>
+      <c r="C23" s="75"/>
+      <c r="D23" s="75"/>
+      <c r="E23" s="91" t="s">
         <v>53</v>
       </c>
-      <c r="F23" s="61"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="62"/>
-      <c r="K23" s="62"/>
-      <c r="L23" s="63"/>
-      <c r="M23" s="92"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
-      <c r="P23" s="93"/>
-      <c r="Q23" s="93"/>
-      <c r="R23" s="94"/>
-      <c r="S23" s="47"/>
-      <c r="T23" s="48"/>
-      <c r="U23" s="48"/>
-      <c r="V23" s="48"/>
-      <c r="W23" s="48"/>
-      <c r="X23" s="48"/>
-      <c r="Y23" s="67"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="38"/>
+      <c r="O23" s="38"/>
+      <c r="P23" s="38"/>
+      <c r="Q23" s="38"/>
+      <c r="R23" s="39"/>
+      <c r="S23" s="79"/>
+      <c r="T23" s="80"/>
+      <c r="U23" s="80"/>
+      <c r="V23" s="80"/>
+      <c r="W23" s="80"/>
+      <c r="X23" s="80"/>
+      <c r="Y23" s="52"/>
       <c r="Z23" s="6"/>
     </row>
     <row r="24" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A24" s="5"/>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="61"/>
-      <c r="G24" s="62"/>
-      <c r="H24" s="62"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="62"/>
-      <c r="K24" s="62"/>
-      <c r="L24" s="63"/>
-      <c r="M24" s="92"/>
-      <c r="N24" s="93"/>
-      <c r="O24" s="93"/>
-      <c r="P24" s="93"/>
-      <c r="Q24" s="93"/>
-      <c r="R24" s="94"/>
-      <c r="S24" s="47"/>
-      <c r="T24" s="48"/>
-      <c r="U24" s="48"/>
-      <c r="V24" s="48"/>
-      <c r="W24" s="48"/>
-      <c r="X24" s="48"/>
-      <c r="Y24" s="67"/>
+      <c r="C24" s="75"/>
+      <c r="D24" s="75"/>
+      <c r="E24" s="92"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="47"/>
+      <c r="H24" s="47"/>
+      <c r="I24" s="47"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="48"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="38"/>
+      <c r="O24" s="38"/>
+      <c r="P24" s="38"/>
+      <c r="Q24" s="38"/>
+      <c r="R24" s="39"/>
+      <c r="S24" s="79"/>
+      <c r="T24" s="80"/>
+      <c r="U24" s="80"/>
+      <c r="V24" s="80"/>
+      <c r="W24" s="80"/>
+      <c r="X24" s="80"/>
+      <c r="Y24" s="52"/>
       <c r="Z24" s="6"/>
     </row>
     <row r="25" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A25" s="5"/>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="93" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="64"/>
-      <c r="G25" s="65"/>
-      <c r="H25" s="65"/>
-      <c r="I25" s="65"/>
-      <c r="J25" s="65"/>
-      <c r="K25" s="65"/>
-      <c r="L25" s="66"/>
-      <c r="M25" s="95"/>
-      <c r="N25" s="96"/>
-      <c r="O25" s="96"/>
-      <c r="P25" s="96"/>
-      <c r="Q25" s="96"/>
-      <c r="R25" s="97"/>
-      <c r="S25" s="49"/>
-      <c r="T25" s="50"/>
-      <c r="U25" s="50"/>
-      <c r="V25" s="50"/>
-      <c r="W25" s="50"/>
-      <c r="X25" s="50"/>
-      <c r="Y25" s="67"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="51"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="41"/>
+      <c r="O25" s="41"/>
+      <c r="P25" s="41"/>
+      <c r="Q25" s="41"/>
+      <c r="R25" s="42"/>
+      <c r="S25" s="81"/>
+      <c r="T25" s="82"/>
+      <c r="U25" s="82"/>
+      <c r="V25" s="82"/>
+      <c r="W25" s="82"/>
+      <c r="X25" s="82"/>
+      <c r="Y25" s="52"/>
       <c r="Z25" s="6"/>
     </row>
     <row r="26" spans="1:26" ht="26" customHeight="1" thickBot="1">
@@ -2177,52 +2213,52 @@
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="94" t="s">
         <v>34</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="95" t="s">
         <v>35</v>
       </c>
-      <c r="H26" s="55"/>
-      <c r="I26" s="51" t="s">
+      <c r="H26" s="62"/>
+      <c r="I26" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="J26" s="52"/>
-      <c r="K26" s="13" t="s">
+      <c r="J26" s="97"/>
+      <c r="K26" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="L26" s="11" t="s">
+      <c r="L26" s="83" t="s">
         <v>37</v>
       </c>
-      <c r="M26" s="11" t="s">
+      <c r="M26" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="N26" s="55"/>
-      <c r="O26" s="53" t="s">
+      <c r="N26" s="62"/>
+      <c r="O26" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="P26" s="54"/>
-      <c r="Q26" s="11" t="s">
+      <c r="P26" s="61"/>
+      <c r="Q26" s="83" t="s">
         <v>40</v>
       </c>
-      <c r="R26" s="15" t="s">
+      <c r="R26" s="100" t="s">
         <v>42</v>
       </c>
-      <c r="S26" s="11" t="s">
+      <c r="S26" s="83" t="s">
         <v>43</v>
       </c>
-      <c r="T26" s="11" t="s">
+      <c r="T26" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="U26" s="51" t="s">
+      <c r="U26" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="V26" s="52"/>
-      <c r="W26" s="37"/>
-      <c r="X26" s="14" t="s">
+      <c r="V26" s="59"/>
+      <c r="W26" s="71"/>
+      <c r="X26" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="Y26" s="67"/>
+      <c r="Y26" s="52"/>
       <c r="Z26" s="6"/>
     </row>
     <row r="27" spans="1:26" ht="26" customHeight="1" thickBot="1">
@@ -2231,66 +2267,66 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
-      <c r="F27" s="22"/>
+      <c r="F27" s="15"/>
       <c r="G27" s="10"/>
-      <c r="H27" s="56"/>
+      <c r="H27" s="63"/>
       <c r="I27" s="10"/>
       <c r="J27" s="10"/>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
-      <c r="M27" s="11" t="s">
+      <c r="M27" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="N27" s="56"/>
-      <c r="O27" s="55"/>
-      <c r="P27" s="55"/>
-      <c r="Q27" s="12" t="s">
+      <c r="N27" s="63"/>
+      <c r="O27" s="62"/>
+      <c r="P27" s="62"/>
+      <c r="Q27" s="99" t="s">
         <v>41</v>
       </c>
-      <c r="R27" s="55"/>
-      <c r="S27" s="55"/>
-      <c r="T27" s="12" t="s">
+      <c r="R27" s="62"/>
+      <c r="S27" s="62"/>
+      <c r="T27" s="99" t="s">
         <v>45</v>
       </c>
-      <c r="U27" s="55"/>
-      <c r="V27" s="55"/>
-      <c r="W27" s="38"/>
-      <c r="X27" s="11" t="s">
+      <c r="U27" s="62"/>
+      <c r="V27" s="62"/>
+      <c r="W27" s="72"/>
+      <c r="X27" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="Y27" s="67"/>
+      <c r="Y27" s="52"/>
       <c r="Z27" s="6"/>
     </row>
     <row r="28" spans="1:26" ht="26" customHeight="1" thickBot="1">
       <c r="A28" s="5"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="E28" s="34"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="25"/>
-      <c r="M28" s="25"/>
-      <c r="N28" s="57"/>
-      <c r="O28" s="57"/>
-      <c r="P28" s="57"/>
-      <c r="Q28" s="25"/>
-      <c r="R28" s="57"/>
-      <c r="S28" s="57"/>
-      <c r="T28" s="25"/>
-      <c r="U28" s="57"/>
-      <c r="V28" s="57"/>
-      <c r="W28" s="39"/>
-      <c r="X28" s="12" t="s">
+      <c r="E28" s="68"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="18"/>
+      <c r="M28" s="18"/>
+      <c r="N28" s="64"/>
+      <c r="O28" s="64"/>
+      <c r="P28" s="64"/>
+      <c r="Q28" s="18"/>
+      <c r="R28" s="64"/>
+      <c r="S28" s="64"/>
+      <c r="T28" s="18"/>
+      <c r="U28" s="64"/>
+      <c r="V28" s="64"/>
+      <c r="W28" s="73"/>
+      <c r="X28" s="99" t="s">
         <v>48</v>
       </c>
-      <c r="Y28" s="67"/>
+      <c r="Y28" s="52"/>
       <c r="Z28" s="6"/>
     </row>
     <row r="29" spans="1:26" ht="24" customHeight="1">
@@ -2299,7 +2335,7 @@
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
-      <c r="F29" s="27"/>
+      <c r="F29" s="20"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -2407,12 +2443,12 @@
     </row>
     <row r="33" spans="1:26" ht="28" customHeight="1">
       <c r="A33" s="5"/>
-      <c r="B33" s="79" t="s">
+      <c r="B33" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="C33" s="80"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="81"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
@@ -2437,10 +2473,10 @@
     </row>
     <row r="34" spans="1:26" ht="28" customHeight="1">
       <c r="A34" s="5"/>
-      <c r="B34" s="82"/>
-      <c r="C34" s="83"/>
-      <c r="D34" s="83"/>
-      <c r="E34" s="84"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="29"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
@@ -2465,10 +2501,10 @@
     </row>
     <row r="35" spans="1:26" ht="28" customHeight="1">
       <c r="A35" s="5"/>
-      <c r="B35" s="82"/>
-      <c r="C35" s="83"/>
-      <c r="D35" s="83"/>
-      <c r="E35" s="84"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="29"/>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
@@ -2493,10 +2529,10 @@
     </row>
     <row r="36" spans="1:26" ht="28" customHeight="1">
       <c r="A36" s="5"/>
-      <c r="B36" s="82"/>
-      <c r="C36" s="83"/>
-      <c r="D36" s="83"/>
-      <c r="E36" s="84"/>
+      <c r="B36" s="27"/>
+      <c r="C36" s="28"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="29"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
@@ -2521,10 +2557,10 @@
     </row>
     <row r="37" spans="1:26" ht="28" customHeight="1" thickBot="1">
       <c r="A37" s="5"/>
-      <c r="B37" s="85"/>
-      <c r="C37" s="86"/>
-      <c r="D37" s="86"/>
-      <c r="E37" s="87"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="32"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
@@ -2577,30 +2613,30 @@
     </row>
     <row r="39" spans="1:26" ht="24" customHeight="1">
       <c r="A39" s="7"/>
-      <c r="B39" s="88"/>
-      <c r="C39" s="88"/>
-      <c r="D39" s="88"/>
-      <c r="E39" s="88"/>
-      <c r="F39" s="88"/>
-      <c r="G39" s="88"/>
-      <c r="H39" s="88"/>
-      <c r="I39" s="88"/>
-      <c r="J39" s="88"/>
-      <c r="K39" s="88"/>
-      <c r="L39" s="88"/>
-      <c r="M39" s="88"/>
-      <c r="N39" s="88"/>
-      <c r="O39" s="88"/>
-      <c r="P39" s="88"/>
-      <c r="Q39" s="88"/>
-      <c r="R39" s="88"/>
-      <c r="S39" s="88"/>
-      <c r="T39" s="88"/>
-      <c r="U39" s="88"/>
-      <c r="V39" s="88"/>
-      <c r="W39" s="88"/>
-      <c r="X39" s="88"/>
-      <c r="Y39" s="88"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="33"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="33"/>
+      <c r="H39" s="33"/>
+      <c r="I39" s="33"/>
+      <c r="J39" s="33"/>
+      <c r="K39" s="33"/>
+      <c r="L39" s="33"/>
+      <c r="M39" s="33"/>
+      <c r="N39" s="33"/>
+      <c r="O39" s="33"/>
+      <c r="P39" s="33"/>
+      <c r="Q39" s="33"/>
+      <c r="R39" s="33"/>
+      <c r="S39" s="33"/>
+      <c r="T39" s="33"/>
+      <c r="U39" s="33"/>
+      <c r="V39" s="33"/>
+      <c r="W39" s="33"/>
+      <c r="X39" s="33"/>
+      <c r="Y39" s="33"/>
       <c r="Z39" s="8"/>
     </row>
     <row r="40" spans="1:26" ht="24" customHeight="1">
@@ -2661,10 +2697,33 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="B3:I5"/>
+    <mergeCell ref="W26:W28"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="C15:D25"/>
+    <mergeCell ref="S15:X25"/>
+    <mergeCell ref="U27:U28"/>
+    <mergeCell ref="V27:V28"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="N26:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="P27:P28"/>
+    <mergeCell ref="R27:R28"/>
+    <mergeCell ref="S27:S28"/>
     <mergeCell ref="B33:E37"/>
     <mergeCell ref="B39:Y39"/>
     <mergeCell ref="M15:R25"/>
-    <mergeCell ref="B3:G5"/>
     <mergeCell ref="F15:L25"/>
     <mergeCell ref="Y8:Y28"/>
     <mergeCell ref="H9:K9"/>
@@ -2677,31 +2736,8 @@
     <mergeCell ref="O26:P26"/>
     <mergeCell ref="U26:V26"/>
     <mergeCell ref="H26:H28"/>
-    <mergeCell ref="N26:N28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="P27:P28"/>
-    <mergeCell ref="R27:R28"/>
-    <mergeCell ref="S27:S28"/>
-    <mergeCell ref="U27:U28"/>
-    <mergeCell ref="V27:V28"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="W26:W28"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="C15:D25"/>
-    <mergeCell ref="S15:X25"/>
   </mergeCells>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="48" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>